<commit_message>
add excel clientes y validacion
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\condominioterrazas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75DB62CC-E136-46C1-9CB3-4A3EBB9CA0F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{389F5CEC-2AC5-4B07-A7DE-C4315CF4B3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{C55A2232-87D0-41ED-9212-52063D1711C8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="20">
   <si>
     <t>DNI</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>joseperez@gmail.com</t>
+  </si>
+  <si>
+    <t>J21</t>
   </si>
 </sst>
 </file>
@@ -475,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD0B8B2F-9FA7-4717-8301-335C9528E270}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="8" width="23.33203125" customWidth="1"/>
@@ -663,6 +666,50 @@
         <v>7</v>
       </c>
     </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>99999999</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8">
+        <v>999999999</v>
+      </c>
+      <c r="E8" s="1"/>
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>99999999</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9">
+        <v>999999999</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{4B8397F1-3A98-4BFF-82AF-19AD53695E25}"/>
@@ -671,6 +718,7 @@
     <hyperlink ref="E5" r:id="rId4" xr:uid="{142A1FD1-C780-49BD-8867-8FC0E372A449}"/>
     <hyperlink ref="E6" r:id="rId5" xr:uid="{76649BCD-034B-48B4-942A-0EAB71E1EB41}"/>
     <hyperlink ref="E7" r:id="rId6" xr:uid="{83DC1F5D-FC83-438D-AEFF-970C3782776F}"/>
+    <hyperlink ref="E9" r:id="rId7" xr:uid="{7CC671D5-0348-4465-A931-8BAD6878A515}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>